<commit_message>
another attempt to update rev hist
</commit_message>
<xml_diff>
--- a/Computations/calc.xlsx
+++ b/Computations/calc.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\01_Engineering\01_Projects\14_450_V_Module_Isol\00_Des\00_CAD\Computations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{B038ABA6-AC84-4795-A87B-DCEFEF122DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{F5395C88-AFED-4F4B-90B6-B20C4B32D6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5F551EED-C412-4F48-9D54-D83EC77118E4}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{5F551EED-C412-4F48-9D54-D83EC77118E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Operating_characteristics" sheetId="8" r:id="rId1"/>
     <sheet name="compensation" sheetId="12" r:id="rId2"/>
-    <sheet name="Sheet9" sheetId="9" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Operating_characteristics!$E$3:$Z$178</definedName>
@@ -110,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="92">
   <si>
     <t>n (L)</t>
   </si>
@@ -140,9 +139,6 @@
   </si>
   <si>
     <t>vout</t>
-  </si>
-  <si>
-    <t>fc &lt; 10 kHz</t>
   </si>
   <si>
     <t>ID</t>
@@ -292,21 +288,6 @@
   </si>
   <si>
     <t>Rd_par</t>
-  </si>
-  <si>
-    <t>Go=</t>
-  </si>
-  <si>
-    <t>Rd</t>
-  </si>
-  <si>
-    <t>Rd + Rup</t>
-  </si>
-  <si>
-    <t>fsw = 50 kHz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frhp = </t>
   </si>
   <si>
     <t>cs [Ω]</t>
@@ -8838,15 +8819,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>131</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:colOff>542925</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>448582</xdr:colOff>
-      <xdr:row>138</xdr:row>
-      <xdr:rowOff>47803</xdr:rowOff>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>305707</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>38278</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -8869,8 +8850,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12077700" y="25631775"/>
-          <a:ext cx="6496957" cy="1276528"/>
+          <a:off x="12544425" y="15487650"/>
+          <a:ext cx="6506482" cy="1276528"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8881,16 +8862,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>99</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>562738</xdr:colOff>
-      <xdr:row>104</xdr:row>
-      <xdr:rowOff>143024</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>19813</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>162074</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -8913,7 +8894,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12001500" y="19459575"/>
+          <a:off x="12573000" y="12011025"/>
           <a:ext cx="5468113" cy="1066949"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8926,15 +8907,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>122</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:colOff>409575</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>41</xdr:col>
-      <xdr:colOff>125023</xdr:colOff>
-      <xdr:row>130</xdr:row>
-      <xdr:rowOff>57353</xdr:rowOff>
+      <xdr:colOff>429823</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>171653</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -8957,8 +8938,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12106275" y="23936325"/>
-          <a:ext cx="8583223" cy="1457528"/>
+          <a:off x="12411075" y="13725525"/>
+          <a:ext cx="8592748" cy="1457528"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8970,15 +8951,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
-      <xdr:row>172</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
-      <xdr:colOff>29451</xdr:colOff>
-      <xdr:row>178</xdr:row>
-      <xdr:rowOff>95423</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>581901</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>123998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -9001,8 +8982,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12573000" y="1485900"/>
-          <a:ext cx="6277851" cy="1238423"/>
+          <a:off x="12430125" y="17516475"/>
+          <a:ext cx="6287376" cy="1238423"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9013,16 +8994,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>581025</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>41</xdr:col>
-      <xdr:colOff>182090</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>48011</xdr:rowOff>
+      <xdr:colOff>10640</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -9045,8 +9026,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12839700" y="1247775"/>
-          <a:ext cx="7992590" cy="2762636"/>
+          <a:off x="12477750" y="9810750"/>
+          <a:ext cx="7992590" cy="1924050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9058,15 +9039,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>590550</xdr:colOff>
-      <xdr:row>174</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>67201</xdr:colOff>
-      <xdr:row>184</xdr:row>
-      <xdr:rowOff>95512</xdr:rowOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>562501</xdr:colOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>181237</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -9089,8 +9070,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14154150" y="37804725"/>
-          <a:ext cx="3772426" cy="1876687"/>
+          <a:off x="12477750" y="19411950"/>
+          <a:ext cx="3781951" cy="1876687"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9346,99 +9327,6 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>66674</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>86243</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>383323</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>134314</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C816F9F-2FE6-93B4-7B39-20A85608365C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="676274" y="276743"/>
-          <a:ext cx="10679849" cy="4429571"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>486529</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>76628</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EC8D8E1-3A8E-D185-DDD5-EB44402F2174}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11668125" y="819150"/>
-          <a:ext cx="5401429" cy="3067478"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -9801,7 +9689,9 @@
     <col min="20" max="20" width="8.28515625" style="9" customWidth="1"/>
     <col min="21" max="21" width="6.140625" customWidth="1"/>
     <col min="22" max="22" width="8.7109375" customWidth="1"/>
-    <col min="26" max="26" width="9.140625" style="29"/>
+    <col min="24" max="25" width="1.5703125" customWidth="1"/>
+    <col min="26" max="26" width="1.5703125" style="29" customWidth="1"/>
+    <col min="27" max="27" width="1.5703125" customWidth="1"/>
     <col min="29" max="29" width="9.140625" style="1"/>
     <col min="30" max="30" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="31" max="16384" width="9.140625" style="1"/>
@@ -9809,66 +9699,66 @@
   <sheetData>
     <row r="3" spans="2:32" s="24" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="22"/>
       <c r="E3" s="22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="22" t="s">
+      <c r="J3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="22" t="s">
+      <c r="K3" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="22" t="s">
-        <v>31</v>
-      </c>
       <c r="L3" s="25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M3" s="22" t="s">
         <v>7</v>
       </c>
       <c r="N3" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="P3" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="R3" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="S3" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="O3" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="P3" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q3" s="22" t="s">
+      <c r="U3" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="R3" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="S3" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="T3" s="25" t="s">
+      <c r="V3" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="U3" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="V3" s="22" t="s">
+      <c r="W3" s="22" t="s">
         <v>35</v>
-      </c>
-      <c r="W3" s="22" t="s">
-        <v>36</v>
       </c>
       <c r="X3" s="22"/>
       <c r="Y3" s="22"/>
@@ -9882,7 +9772,7 @@
     </row>
     <row r="4" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="13">
         <f>3.54*0.000001</f>
@@ -9968,7 +9858,7 @@
     </row>
     <row r="5" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="14">
         <f>1453*0.000001</f>
@@ -10973,7 +10863,7 @@
     </row>
     <row r="17" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B17" s="37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17" s="38"/>
       <c r="D17" s="11"/>
@@ -11056,7 +10946,7 @@
     </row>
     <row r="18" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B18" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" s="17">
         <f>50*1000</f>
@@ -11143,7 +11033,7 @@
     </row>
     <row r="19" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B19" s="19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="5">
         <v>0.45</v>
@@ -11229,7 +11119,7 @@
     </row>
     <row r="20" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B20" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" s="14">
         <f>10*0.000001</f>
@@ -11315,7 +11205,7 @@
     </row>
     <row r="21" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B21" s="18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C21" s="5">
         <v>0.75</v>
@@ -11400,7 +11290,7 @@
     </row>
     <row r="22" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B22" s="20" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C22" s="39">
         <v>1.2999999999999999E-2</v>
@@ -23666,18 +23556,18 @@
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="M3" s="8"/>
     </row>
@@ -23686,7 +23576,7 @@
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="30" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M5" s="8"/>
     </row>
@@ -23695,7 +23585,7 @@
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C7" s="40">
         <v>1.0000000000000001E-5</v>
@@ -23711,34 +23601,34 @@
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="M7" s="8"/>
       <c r="N7" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="O7" s="8" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="Q7" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C8" s="8">
         <v>1</v>
@@ -23788,7 +23678,7 @@
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C9" s="8">
         <v>100</v>
@@ -23839,7 +23729,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C10" s="8">
         <v>70</v>
@@ -23889,7 +23779,7 @@
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C11" s="11">
         <f>C9^2/C10</f>
@@ -23943,7 +23833,7 @@
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C12" s="8">
         <f>C10/C9</f>
@@ -24081,7 +23971,7 @@
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C15" s="1">
         <f>1/(2*PI()*C7*C11)</f>
@@ -24126,7 +24016,7 @@
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C16" s="1">
         <f>1/(2*PI()*C7*C8)</f>
@@ -24158,7 +24048,7 @@
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C17" s="8">
         <f>C11*C12</f>
@@ -24182,7 +24072,7 @@
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C18" s="1">
         <f>20*LOG(C17)</f>
@@ -24214,45 +24104,45 @@
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21" s="30" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="M21" s="8"/>
     </row>
     <row r="22" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C22" s="8" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="J22" s="8"/>
       <c r="L22" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="M22" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="M22" s="8" t="s">
-        <v>96</v>
       </c>
       <c r="N22" s="8"/>
       <c r="P22" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q22" s="8" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="R22" s="8"/>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C23" s="8">
         <v>480000</v>
@@ -24302,7 +24192,7 @@
     </row>
     <row r="24" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C24" s="9">
         <v>3200</v>
@@ -24352,7 +24242,7 @@
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C25" s="9">
         <f>1/(1/C23+1/C24)</f>
@@ -24405,7 +24295,7 @@
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C26" s="34">
         <f>C24/(C24+C23)</f>
@@ -24458,7 +24348,7 @@
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C27" s="9">
         <v>6.6666600000000004E-13</v>
@@ -24499,7 +24389,7 @@
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C28" s="9">
         <v>1E-8</v>
@@ -24537,7 +24427,7 @@
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C29" s="9">
         <v>15000000</v>
@@ -24559,7 +24449,7 @@
     </row>
     <row r="31" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C31" s="1">
         <f>1/(2*PI()*C29*C28)</f>
@@ -24576,7 +24466,7 @@
     </row>
     <row r="32" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C32" s="11">
         <f>1/(2*PI()*C29*C27)</f>
@@ -24594,7 +24484,7 @@
     </row>
     <row r="33" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C33" s="1">
         <f>C29/C25*C26</f>
@@ -24612,7 +24502,7 @@
     </row>
     <row r="34" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C34" s="1">
         <f>20*LOG(C33)</f>
@@ -24647,50 +24537,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8097CF1-D74A-4106-A621-545AE6035C82}">
-  <dimension ref="B25:U28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="T25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="T26" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>49</v>
-      </c>
-      <c r="C27" t="s">
-        <v>50</v>
-      </c>
-      <c r="T27" t="s">
-        <v>53</v>
-      </c>
-      <c r="U27">
-        <f>(1-0.45)^2*208/(2*PI()*0.45*0.05^2*3.54*0.000001)</f>
-        <v>2514508228.3344774</v>
-      </c>
-    </row>
-    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97643BEB-A645-498A-B952-4DE4DC670158}">
   <dimension ref="B2:Z36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -24702,7 +24548,7 @@
   <sheetData>
     <row r="2" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B2" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="8">
         <v>550</v>
@@ -24714,10 +24560,10 @@
         <v>8</v>
       </c>
       <c r="G2" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="8" t="s">
         <v>44</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>45</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>9</v>
@@ -24737,7 +24583,7 @@
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C3" s="8">
         <v>170</v>
@@ -24772,7 +24618,7 @@
     </row>
     <row r="4" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4" s="8">
         <v>2.5</v>
@@ -24807,13 +24653,13 @@
     </row>
     <row r="5" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="8">
         <v>480</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
@@ -24868,14 +24714,14 @@
     </row>
     <row r="7" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="10">
         <f>C4/((C2-C4)/C5)</f>
         <v>2.1917808219178081</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F7" s="10">
         <v>2</v>
@@ -24904,14 +24750,14 @@
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="10">
         <f>C4/((C3-C4)/C5)</f>
         <v>7.1641791044776122</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F8" s="10">
         <v>2.5</v>
@@ -24940,14 +24786,14 @@
     </row>
     <row r="9" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="10">
         <f>C8-C7</f>
         <v>4.9723982825598041</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F9" s="10">
         <v>3</v>
@@ -24976,13 +24822,13 @@
     </row>
     <row r="10" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="8">
         <v>2.2000000000000002</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F10" s="10">
         <v>3.5</v>
@@ -25011,13 +24857,13 @@
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" s="11">
         <v>1000</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F11" s="10">
         <v>4</v>
@@ -25098,12 +24944,12 @@
     </row>
     <row r="19" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F21" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="6:14" x14ac:dyDescent="0.25">
@@ -25113,7 +24959,7 @@
     </row>
     <row r="23" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F23" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
@@ -25121,22 +24967,22 @@
     </row>
     <row r="24" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F24" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F25" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F26" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F27" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="12:14" x14ac:dyDescent="0.25">

</xml_diff>